<commit_message>
COACH GUIDE tab: team/coach names, pull % on real chances with bands, typical pull timing, plain-language PP explainer; profiles builder script + RUNBOOK entry
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012si27ZfLSnpNPfN3rGmhCN
</commit_message>
<xml_diff>
--- a/live_model/lines_table_30s.xlsx
+++ b/live_model/lines_table_30s.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LINES" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO USE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COACH GUIDE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOW TO USE" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LINES'!$A$2:$L$452</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'COACH GUIDE'!$A$2:$H$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +48,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00999999"/>
     </font>
   </fonts>
   <fills count="6">
@@ -93,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -106,6 +112,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -25810,75 +25821,1901 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>WHO PULLS, AND WHEN — pull %% counted on REAL chances only (gap still 3, net available, no penalty problem, inside the pull zone). League average on a real chance: 64%%. 5v5 pulls happen around 4:19 left; power-play pulls around 3:33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Pull % (real chances)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Range (95%)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Typical pull time left</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>LINES row to use</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Joel Quenneville</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>58%-100%</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>3:53</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>small sample (3 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Greg Cronin (former)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>2%-69%</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>5v5: very passive | on PP: league avg</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>PP-ONLY puller; only pulls ON the power play -&gt; see HOW TO USE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Marco Sturm</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>1%-99%</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>small sample (2 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Joe Sacco (former)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>71%-100%</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>4:05</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>pulls EVERY real chance so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Lindy Ruff</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>63%-100%</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>2:46</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Rod Brind'Amour</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>31%-98%</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>4:13</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Rick Bowness</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>0/0</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>small sample (0 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Dean Evason (former)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>6/11</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>27%-81%</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>4:47</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Ryan Huska</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>0%-33%</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>rarely pulls</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Jeff Blashill</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>22%-95%</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>5:22</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Anders Sorensen (former)</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>0%-34%</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>small sample (4 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Luke Richardson (former)</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>0%-74%</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>small sample (1 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Jared Bednar</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>9/9</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>82%-100%</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>3:49</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>1.85 very aggressive</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>pulls EVERY real chance so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Glen Gulutzan</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>50%-100%</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>4:28</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Todd McLellan</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>2/8</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>0%-56%</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>5v5: very passive | on PP: league avg</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>PP-ONLY puller; only pulls ON the power play -&gt; see HOW TO USE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Derek Lalonde (former)</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>33%-100%</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>small sample (4 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Kris Knoblauch</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>60%-100%</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Paul Maurice</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>7/12</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>32%-84%</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>5:15</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>D.J. Smith</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>26%-100%</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>small sample (1 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Jim Hiller (former)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>4/7</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>24%-89%</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>3:13</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>John Hynes</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>7/11</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>36%-89%</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>3:19</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Martin St. Louis</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>6/11</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>27%-81%</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>4:38</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Sheldon Keefe</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>8/15</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>29%-77%</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>6:05</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Andrew Brunette</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>4/12</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>10%-60%</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>4:38</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Peter DeBoer</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>1%-99%</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>small sample (2 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Patrick Roy (former)</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>12/14</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>65%-100%</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>7:37</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Mike Sullivan</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>6/10</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>31%-87%</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>5:14</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Peter Laviolette (former)</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>58%-100%</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>3:40</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>small sample (3 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Travis Green</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>63%-100%</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>4:11</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Rick Tocchet</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>5/7</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>38%-99%</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>3:52</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Brad Shaw (former)</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>0%-74%</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>small sample (1 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Dan Muse</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>80%-100%</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>5:19</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>pulls EVERY real chance so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Lane Lambert</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>31%-98%</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>3:34</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Dan Bylsma (former)</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>7/7</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>78%-100%</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>3:58</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>pulls EVERY real chance so far</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Ryan Warsofsky</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>5/11</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>19%-73%</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>3:25</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Jim Montgomery</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>0.571</v>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>4/7</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>24%-89%</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>6:23</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Drew Bannister (former)</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>0/0</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>small sample (0 chances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Jon Cooper</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>67%-100%</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>4:20</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Craig Berube</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>15/19</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>60%-95%</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>4:19</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>1.30 aggressive</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>AndrÃ© Tourigny</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>2%-69%</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Adam Foote</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>8/12</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>40%-90%</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>4:59</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>John Tortorella</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>2/8</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>0%-56%</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>~4:19 (league, few pulls)</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>5v5: very passive | on PP: league avg</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>PP-ONLY puller; only pulls ON the power play -&gt; see HOW TO USE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Bruce Cassidy (former)</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>7/11</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>36%-89%</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Scott Arniel</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>6/8</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>44%-100%</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>5:01</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>1.00 league avg</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Spencer Carbery</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>3/8</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>9%-69%</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>2:26</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>0.80 passive</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:H47"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C3:C47">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.64"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>HOW TO USE</t>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>HOW TO USE (3 steps)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>1. Filter 'Situation' to the current state and 'Coach type' to the trailing coach's tier (COACHES tab of the calculator).</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>1. COACH GUIDE tab: find the trailing team -&gt; current coach (bold). Read his pull % on real chances, his typical pull time, and which LINES row to use.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>2. Find the time remaining (rows are 30-second steps; for in-between times use the calculator, which takes any mm:ss).</t>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>2. LINES tab: filter 'Situation' + 'Coach type' to what the guide told you, find the time remaining.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>3. The TRUE line shows the fair price (0% EV, break-even). The line @10% is the worst price at which the bet still clears +10% EV. Better than @10% = bet; worse = pass.</t>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>3. TRUE line = fair price (break-even). Line @10% = worst price that still pays +10%% EV. Book offering better than the @10%% number = bet. Worse = pass.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr"/>
+      <c r="A5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>THE POWER-PLAY THING, PLAINLY:</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>'Net in — POWER PLAY' rows = the team that is DOWN 3 has a power play. Pulling the goalie then gives 6 skaters vs 4 — the best pull there is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Every coach pulls more on the PP (league: ~4x). But four coaches — Tortorella, McLellan, Cronin, Huska — basically ONLY pull then:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>two full seasons, ZERO 5v5 pulls between them, yet on the PP they pull at league rate or higher.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>So for those four: down 3 at 5v5 -&gt; assume NO pull is coming (very passive rows). They get a power play under ~7:00 -&gt; switch to the</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>POWER PLAY rows at league-avg aggression. That is the moment their pull (and your over/-3.5 value) actually arrives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Reading lines: -196 means bet only at -196 or better (e.g. -180, -150, +110). +150 means +150 or longer.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Coach type: multiplier applied to pull aggressiveness. 1.00 = league average. Bednar-class ~1.3-1.85; PP-only coaches (Tortorella, McLellan, Cronin, Huska): use 'Net in — POWER PLAY' rows when they have a PP, else assume near-zero pull.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Pull % caveat: 9/9 does NOT mean a guaranteed 100%% — small samples, read the Range column (9/9 -&gt; can't rule out ~82%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Colors: green = likely, red = unlikely. Blue rows = trailing team on power play. Orange rows = net already empty.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Provenance: dense MC grid n=30k seed 7, fits both seasons, blind-validated 25-26 (leader TT +30.7% ROI at these lines).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Rebuild (cheap session): python3 hockeycore/io/build_lines_table.py</t>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>NO-GO for real money (Seb ruling). Leader market = Overs only. Provenance: MC grid n=30k seed 7, blind-validated 25-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Rebuild (cheap session): python3 hockeycore/io/build_lines_table.py  (needs data/derived/coach_profiles.json)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
5v5-only pull ledger is now THE number (Seb: PP pulls not bettable — lines vanish on PP). PP-only four = 0/23 at 5v5 combined; Keefe 53->38, Hiller 57->25. Guide + explainer reframed; EV-only pull timing
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012si27ZfLSnpNPfN3rGmhCN
</commit_message>
<xml_diff>
--- a/live_model/lines_table_30s.xlsx
+++ b/live_model/lines_table_30s.xlsx
@@ -25837,7 +25837,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WHO PULLS, AND WHEN — pull %% counted on REAL chances only (gap still 3, net available, no penalty problem, inside the pull zone). League average on a real chance: 64%%. 5v5 pulls happen around 4:19 left; power-play pulls around 3:33.</t>
+          <t>WHO PULLS, AND WHEN — pull % counted on clean 5v5 chances ONLY (gap still 3, net available, 5-on-5, inside the pull zone). PP pulls are EXCLUDED on purpose: no line is available once a PP starts, so only 5v5 willingness is bettable. 5v5 pulls happen around 4:19 left.</t>
         </is>
       </c>
     </row>
@@ -25854,7 +25854,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Pull % (real chances)</t>
+          <t>5v5 pull % (bettable)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -25935,16 +25935,16 @@
         </is>
       </c>
       <c r="C4" s="12" t="n">
-        <v>0.333</v>
+        <v>0</v>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>0/3</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>2%-69%</t>
+          <t>0%-42%</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
@@ -25954,12 +25954,12 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>5v5: very passive | on PP: league avg</t>
+          <t>very passive (treat as no-pull)</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>PP-ONLY puller; only pulls ON the power play -&gt; see HOW TO USE</t>
+          <t>pulls ONLY on PP (0% at 5v5 = the bettable number); small sample (3 chances)</t>
         </is>
       </c>
     </row>
@@ -25975,16 +25975,16 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>1%-99%</t>
+          <t>26%-100%</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -25999,7 +25999,7 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>small sample (2 chances)</t>
+          <t>small sample (1 chances)</t>
         </is>
       </c>
     </row>
@@ -26039,7 +26039,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>pulls EVERY real chance so far</t>
+          <t>pulls EVERY clean 5v5 chance so far</t>
         </is>
       </c>
     </row>
@@ -26055,21 +26055,21 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.846</v>
+        <v>0.8</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>8/10</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>63%-100%</t>
+          <t>54%-100%</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>2:46</t>
+          <t>4:24</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -26077,7 +26077,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>+3 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -26091,21 +26095,21 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>0.667</v>
+        <v>0.5</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>31%-98%</t>
+          <t>10%-90%</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>4:13</t>
+          <t>~4:19 (league, few pulls)</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -26113,7 +26117,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>small sample (4 chances); +2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -26165,16 +26173,16 @@
         </is>
       </c>
       <c r="C10" s="12" t="n">
-        <v>0.545</v>
+        <v>0.429</v>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>3/7</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>27%-81%</t>
+          <t>11%-76%</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -26187,7 +26195,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>+3 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -26201,16 +26213,16 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>1/10</t>
+          <t>0/8</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>0%-33%</t>
+          <t>0%-20%</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -26225,7 +26237,7 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>rarely pulls</t>
+          <t>rarely pulls; +1 PP pulls (excluded above)</t>
         </is>
       </c>
     </row>
@@ -26281,12 +26293,12 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>0/4</t>
+          <t>0/3</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>0%-34%</t>
+          <t>0%-42%</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -26301,7 +26313,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>small sample (4 chances)</t>
+          <t>small sample (3 chances)</t>
         </is>
       </c>
     </row>
@@ -26316,17 +26328,15 @@
           <t>Luke Richardson (former)</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
-        <v>0</v>
-      </c>
+      <c r="C14" s="12" t="n"/>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>0/0</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>0%-74%</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -26341,7 +26351,7 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>small sample (1 chances)</t>
+          <t>small sample (0 chances)</t>
         </is>
       </c>
     </row>
@@ -26361,17 +26371,17 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>9/9</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>82%-100%</t>
+          <t>75%-100%</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>3:49</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -26381,7 +26391,7 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>pulls EVERY real chance so far</t>
+          <t>pulls EVERY clean 5v5 chance so far; +3 PP pulls (excluded above)</t>
         </is>
       </c>
     </row>
@@ -26397,16 +26407,16 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>0.833</v>
+        <v>0.75</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>50%-100%</t>
+          <t>33%-100%</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -26419,7 +26429,11 @@
           <t>1.30 aggressive</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr"/>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>small sample (4 chances); +2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -26433,16 +26447,16 @@
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>0%-56%</t>
+          <t>0%-25%</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -26452,12 +26466,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>5v5: very passive | on PP: league avg</t>
+          <t>very passive (treat as no-pull)</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>PP-ONLY puller; only pulls ON the power play -&gt; see HOW TO USE</t>
+          <t>pulls ONLY on PP (0% at 5v5 = the bettable number)</t>
         </is>
       </c>
     </row>
@@ -26549,16 +26563,16 @@
         </is>
       </c>
       <c r="C20" s="10" t="n">
-        <v>0.583</v>
+        <v>0.444</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>7/12</t>
+          <t>4/9</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>32%-84%</t>
+          <t>16%-74%</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -26571,7 +26585,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>+3 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -26625,21 +26643,21 @@
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>0.571</v>
+        <v>0.25</v>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>4/7</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>24%-89%</t>
+          <t>0%-67%</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>3:13</t>
+          <t>~4:19 (league, few pulls)</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -26647,7 +26665,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr"/>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>small sample (4 chances); +3 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -26661,16 +26683,16 @@
         </is>
       </c>
       <c r="C23" s="10" t="n">
-        <v>0.636</v>
+        <v>0.625</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>36%-89%</t>
+          <t>31%-91%</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -26683,7 +26705,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>+2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -26697,16 +26723,16 @@
         </is>
       </c>
       <c r="C24" s="10" t="n">
-        <v>0.545</v>
+        <v>0.6</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>6/11</t>
+          <t>6/10</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>27%-81%</t>
+          <t>31%-87%</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -26733,21 +26759,21 @@
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>0.533</v>
+        <v>0.385</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>8/15</t>
+          <t>5/13</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>29%-77%</t>
+          <t>15%-64%</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>6:05</t>
+          <t>6:15</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -26755,7 +26781,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr"/>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>+3 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -26769,16 +26799,16 @@
         </is>
       </c>
       <c r="C26" s="10" t="n">
-        <v>0.333</v>
+        <v>0.273</v>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>4/12</t>
+          <t>3/11</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>10%-60%</t>
+          <t>4%-54%</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -26791,7 +26821,11 @@
           <t>0.80 passive</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>+1 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -26881,21 +26915,21 @@
         </is>
       </c>
       <c r="C29" s="10" t="n">
-        <v>0.6</v>
+        <v>0.625</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>6/10</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>31%-87%</t>
+          <t>31%-91%</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>5:14</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -26903,7 +26937,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H29" s="8" t="inlineStr"/>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>+1 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -26957,21 +26995,21 @@
         </is>
       </c>
       <c r="C31" s="10" t="n">
-        <v>0.846</v>
+        <v>0.625</v>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>5/8</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>63%-100%</t>
+          <t>31%-91%</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>4:11</t>
+          <t>4:54</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -26979,7 +27017,11 @@
           <t>1.30 aggressive</t>
         </is>
       </c>
-      <c r="H31" s="8" t="inlineStr"/>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>+6 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -26993,21 +27035,21 @@
         </is>
       </c>
       <c r="C32" s="10" t="n">
-        <v>0.714</v>
+        <v>0.75</v>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>5/7</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>38%-99%</t>
+          <t>33%-100%</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>3:52</t>
+          <t>3:43</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
@@ -27015,7 +27057,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr"/>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>small sample (4 chances); +2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -27073,17 +27119,17 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>8/8</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>80%-100%</t>
+          <t>71%-100%</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>5:19</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -27093,7 +27139,7 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>pulls EVERY real chance so far</t>
+          <t>pulls EVERY clean 5v5 chance so far; +3 PP pulls (excluded above)</t>
         </is>
       </c>
     </row>
@@ -27109,21 +27155,21 @@
         </is>
       </c>
       <c r="C35" s="10" t="n">
-        <v>0.667</v>
+        <v>0.75</v>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>31%-98%</t>
+          <t>33%-100%</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
-          <t>3:34</t>
+          <t>2:53</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -27131,7 +27177,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr"/>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>small sample (4 chances); +1 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -27149,12 +27199,12 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>7/7</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>78%-100%</t>
+          <t>75%-100%</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
@@ -27169,7 +27219,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>pulls EVERY real chance so far</t>
+          <t>pulls EVERY clean 5v5 chance so far; +1 PP pulls (excluded above)</t>
         </is>
       </c>
     </row>
@@ -27185,21 +27235,21 @@
         </is>
       </c>
       <c r="C37" s="10" t="n">
-        <v>0.455</v>
+        <v>0.3</v>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>5/11</t>
+          <t>3/10</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>19%-73%</t>
+          <t>6%-58%</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>3:25</t>
+          <t>4:39</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
@@ -27207,7 +27257,11 @@
           <t>0.80 passive</t>
         </is>
       </c>
-      <c r="H37" s="8" t="inlineStr"/>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>+2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -27221,16 +27275,16 @@
         </is>
       </c>
       <c r="C38" s="10" t="n">
-        <v>0.571</v>
+        <v>0.667</v>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>4/7</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>24%-89%</t>
+          <t>31%-98%</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -27295,21 +27349,21 @@
         </is>
       </c>
       <c r="C40" s="10" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>9/10</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>67%-100%</t>
+          <t>66%-100%</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>4:20</t>
+          <t>5:01</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -27317,7 +27371,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr"/>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>small sample (4 chances); +5 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -27331,16 +27389,16 @@
         </is>
       </c>
       <c r="C41" s="10" t="n">
-        <v>0.789</v>
+        <v>0.765</v>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>15/19</t>
+          <t>13/17</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>60%-95%</t>
+          <t>56%-94%</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -27353,7 +27411,11 @@
           <t>1.30 aggressive</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr"/>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>+2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -27367,16 +27429,16 @@
         </is>
       </c>
       <c r="C42" s="10" t="n">
-        <v>0.333</v>
+        <v>0.5</v>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>2%-69%</t>
+          <t>10%-90%</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -27389,7 +27451,11 @@
           <t>0.80 passive</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr"/>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>small sample (4 chances)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
@@ -27439,16 +27505,16 @@
         </is>
       </c>
       <c r="C44" s="10" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>0%-56%</t>
+          <t>0%-25%</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -27458,12 +27524,12 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>5v5: very passive | on PP: league avg</t>
+          <t>very passive (treat as no-pull)</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>PP-ONLY puller; only pulls ON the power play -&gt; see HOW TO USE</t>
+          <t>pulls ONLY on PP (0% at 5v5 = the bettable number)</t>
         </is>
       </c>
     </row>
@@ -27479,21 +27545,21 @@
         </is>
       </c>
       <c r="C45" s="12" t="n">
-        <v>0.636</v>
+        <v>0.714</v>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>7/11</t>
+          <t>5/7</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>36%-89%</t>
+          <t>38%-99%</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>4:04</t>
+          <t>4:48</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
@@ -27501,7 +27567,11 @@
           <t>1.00 league avg</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr"/>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>+2 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -27551,21 +27621,21 @@
         </is>
       </c>
       <c r="C47" s="10" t="n">
-        <v>0.375</v>
+        <v>0.4</v>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>9%-69%</t>
+          <t>5%-78%</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>2:26</t>
+          <t>~4:19 (league, few pulls)</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -27573,7 +27643,11 @@
           <t>0.80 passive</t>
         </is>
       </c>
-      <c r="H47" s="8" t="inlineStr"/>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>+1 PP pulls (excluded above)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:H47"/>
@@ -27602,7 +27676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -27642,78 +27716,85 @@
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>THE POWER-PLAY THING, PLAINLY:</t>
+          <t>WHY PP PULLS ARE SHOWN SEPARATELY (NOT a betting trigger):</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>'Net in — POWER PLAY' rows = the team that is DOWN 3 has a power play. Pulling the goalie then gives 6 skaters vs 4 — the best pull there is.</t>
+          <t>You will never get a line once the trailing team is on a power play — books pull the market. So PP pulls can never be bet on.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Every coach pulls more on the PP (league: ~4x). But four coaches — Tortorella, McLellan, Cronin, Huska — basically ONLY pull then:</t>
+          <t>They matter for one reason: getting a coach's TRUE 5v5 willingness right. Four coaches (Tortorella, McLellan, Cronin, Huska)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>two full seasons, ZERO 5v5 pulls between them, yet on the PP they pull at league rate or higher.</t>
+          <t>look like occasional pullers in raw stats, but every one of their pulls came on a PP. Counting those would trick you into</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>So for those four: down 3 at 5v5 -&gt; assume NO pull is coming (very passive rows). They get a power play under ~7:00 -&gt; switch to the</t>
+          <t>pricing some 5v5 pull chance for them. The truth: at 5v5 they are 0-for-23 combined on clean chances — treat as no-pull teams.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>POWER PLAY rows at league-avg aggression. That is the moment their pull (and your over/-3.5 value) actually arrives.</t>
+          <t>Same logic everywhere: the guide's pull % counts ONLY clean 5v5 chances, so e.g. Keefe is 38% (not the 53% raw) and</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr"/>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Bednar's 100% is 6/6 pure 5v5. The POWER PLAY rows stay in the LINES tab for understanding the game, not for betting.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>Reading lines: -196 means bet only at -196 or better (e.g. -180, -150, +110). +150 means +150 or longer.</t>
-        </is>
-      </c>
+      <c r="A13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Pull % caveat: 9/9 does NOT mean a guaranteed 100%% — small samples, read the Range column (9/9 -&gt; can't rule out ~82%).</t>
+          <t>Reading lines: -196 means bet only at -196 or better (e.g. -180, -150, +110). +150 means +150 or longer.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Colors: green = likely, red = unlikely. Blue rows = trailing team on power play. Orange rows = net already empty.</t>
+          <t>Pull % caveat: 9/9 does NOT mean a guaranteed 100%% — small samples, read the Range column (9/9 -&gt; can't rule out ~82%).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>NO-GO for real money (Seb ruling). Leader market = Overs only. Provenance: MC grid n=30k seed 7, blind-validated 25-26.</t>
+          <t>Colors: green = likely, red = unlikely. Blue rows = trailing team on power play. Orange rows = net already empty.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>NO-GO for real money (Seb ruling). Leader market = Overs only. Provenance: MC grid n=30k seed 7, blind-validated 25-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Rebuild (cheap session): python3 hockeycore/io/build_lines_table.py  (needs data/derived/coach_profiles.json)</t>
         </is>

</xml_diff>